<commit_message>
Deployed dba5279 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Seelenbändiger.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Seelenbändiger.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FDA599B-A755-40F7-B6B6-BC2AD48B2C14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9B2ADC-62D0-43E8-985A-43CBB9A5F62A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="130">
   <si>
     <t>Diese Sprache leitet die Sprache der Hölle weiter, da die Seelenbändiger diese gesprochen hatten, wie sie zusammen in einem Stamm gelebt hatten. Die späteren Nationen geführt durch die Bändiger entickelten die Sprachen weiter, die von Naitro'Nai wurde marziallischer, vorallem in der Hölle, als sich Bedeutungen start änderten.</t>
   </si>
@@ -379,6 +379,42 @@
   </si>
   <si>
     <t>Orin</t>
+  </si>
+  <si>
+    <t>Plague</t>
+  </si>
+  <si>
+    <t>Shaik</t>
+  </si>
+  <si>
+    <t>Sun</t>
+  </si>
+  <si>
+    <t>Moon</t>
+  </si>
+  <si>
+    <t>Dilarii</t>
+  </si>
+  <si>
+    <t>Darkness</t>
+  </si>
+  <si>
+    <t>Trelar</t>
+  </si>
+  <si>
+    <t>Tre</t>
+  </si>
+  <si>
+    <t>Spike</t>
+  </si>
+  <si>
+    <t>Meridor</t>
+  </si>
+  <si>
+    <t>Sorii</t>
+  </si>
+  <si>
+    <t>Wheat</t>
   </si>
 </sst>
 </file>
@@ -696,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B72"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1212,6 +1248,54 @@
         <v>116</v>
       </c>
     </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>119</v>
+      </c>
+      <c r="B67" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>122</v>
+      </c>
+      <c r="B68" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>124</v>
+      </c>
+      <c r="B69" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>125</v>
+      </c>
+      <c r="B70" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>127</v>
+      </c>
+      <c r="B71" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>128</v>
+      </c>
+      <c r="B72" t="s">
+        <v>129</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Deployed b99b060 with MkDocs version: 1.6.1
</commit_message>
<xml_diff>
--- a/Buch Bayrische Nächte/Sprache der Seelenbändiger.xlsx
+++ b/Buch Bayrische Nächte/Sprache der Seelenbändiger.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julian Dauner\Documents\GitHub\pnpWiki\docs\Buch Bayrische Nächte\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF9B2ADC-62D0-43E8-985A-43CBB9A5F62A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C641AC3F-C8E7-4B03-B6E1-B292EEF31CC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="5205" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="132">
   <si>
     <t>Diese Sprache leitet die Sprache der Hölle weiter, da die Seelenbändiger diese gesprochen hatten, wie sie zusammen in einem Stamm gelebt hatten. Die späteren Nationen geführt durch die Bändiger entickelten die Sprachen weiter, die von Naitro'Nai wurde marziallischer, vorallem in der Hölle, als sich Bedeutungen start änderten.</t>
   </si>
@@ -315,9 +315,6 @@
     <t>Fire</t>
   </si>
   <si>
-    <t>Animal</t>
-  </si>
-  <si>
     <t>Body</t>
   </si>
   <si>
@@ -415,6 +412,15 @@
   </si>
   <si>
     <t>Wheat</t>
+  </si>
+  <si>
+    <t>Nel</t>
+  </si>
+  <si>
+    <t>Flora</t>
+  </si>
+  <si>
+    <t>Fauna</t>
   </si>
 </sst>
 </file>
@@ -732,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B72"/>
+  <dimension ref="A1:B73"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -1146,7 +1152,7 @@
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B54" t="s">
         <v>92</v>
@@ -1154,7 +1160,7 @@
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B55" t="s">
         <v>93</v>
@@ -1162,7 +1168,7 @@
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B56" t="s">
         <v>94</v>
@@ -1170,7 +1176,7 @@
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B57" t="s">
         <v>95</v>
@@ -1178,122 +1184,130 @@
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B58" t="s">
-        <v>96</v>
+        <v>131</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B59" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B60" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B61" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B62" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B63" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B64" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B65" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B66" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B67" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B68" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B69" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B70" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B71" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
+        <v>127</v>
+      </c>
+      <c r="B72" t="s">
         <v>128</v>
       </c>
-      <c r="B72" t="s">
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
         <v>129</v>
+      </c>
+      <c r="B73" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>

</xml_diff>